<commit_message>
Monthly update: extend CPI series to 2026-03
- Add gasoline/kerosene subsidy entries for 2026-03 (METI PDF, emergency mitigation period)
- Refresh BOJ Excel and regenerate output charts
- 2026-03 results: core 2.54%/BOJ 2.5%, core_core 2.60%/BOJ 2.6%, BOJ-core 1.74%/BOJ 1.7% (差<0.05pp)

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/boj/cpi_core_indicators.xlsx
+++ b/data/boj/cpi_core_indicators.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F3B9D8-0507-43DC-8E55-65FC13CE7E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FAAA0F8-3929-4EA3-B0DF-A1847310DBB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -800,7 +800,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AY307"/>
+  <dimension ref="A1:AY308"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.2" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="7"/>
@@ -13013,19 +13013,19 @@
         <v>2026.1</v>
       </c>
       <c r="AU166" s="6">
-        <v>2.2000000000000002</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="AV166" s="6">
-        <v>2.8</v>
+        <v>2.7</v>
       </c>
       <c r="AW166" s="6">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
       <c r="AX166" s="6">
-        <v>0.72316930515018751</v>
+        <v>0.7059339935492347</v>
       </c>
       <c r="AY166" s="6">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="167" spans="1:51" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -19804,6 +19804,46 @@
       <c r="AG307" s="6"/>
       <c r="AH307" s="6"/>
     </row>
+    <row r="308" spans="1:34" x14ac:dyDescent="0.2">
+      <c r="A308" s="7">
+        <v>46082</v>
+      </c>
+      <c r="B308" s="6">
+        <v>2.5</v>
+      </c>
+      <c r="C308" s="6"/>
+      <c r="E308" s="6">
+        <v>2.6</v>
+      </c>
+      <c r="F308" s="6"/>
+      <c r="H308" s="6">
+        <v>1.7</v>
+      </c>
+      <c r="I308" s="6"/>
+      <c r="K308" s="6">
+        <v>1.6409894265293685</v>
+      </c>
+      <c r="L308" s="6"/>
+      <c r="Q308" s="6">
+        <v>0.67146337034732906</v>
+      </c>
+      <c r="R308" s="6"/>
+      <c r="W308" s="6">
+        <v>1.4</v>
+      </c>
+      <c r="AC308" s="6">
+        <v>73.946360153256705</v>
+      </c>
+      <c r="AD308" s="6">
+        <v>21.264367816091951</v>
+      </c>
+      <c r="AE308" s="6">
+        <v>52.681992337164758</v>
+      </c>
+      <c r="AF308" s="6"/>
+      <c r="AG308" s="6"/>
+      <c r="AH308" s="6"/>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.39370078740157483" right="0.39370078740157483" top="0.39370078740157483" bottom="0.39370078740157483" header="0.31496062992125984" footer="0.31496062992125984"/>

</xml_diff>